<commit_message>
removing some uneccesary dirs and files
</commit_message>
<xml_diff>
--- a/largescaletesting/input_data.xlsx
+++ b/largescaletesting/input_data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10824"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11110"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/khaniyau2/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/paramdesai/research/ComputationalBiochemistry/Splitting-Ig-Folds_new/largescaletesting/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{695275E6-F855-5D4A-B35B-71D7D60AEE3E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78842132-7521-9E4F-8167-BB6F54BB5908}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="760" windowWidth="27640" windowHeight="16940" activeTab="1" xr2:uid="{347B289A-C670-374C-BA56-7E86338DD0B9}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17720" xr2:uid="{347B289A-C670-374C-BA56-7E86338DD0B9}"/>
   </bookViews>
   <sheets>
     <sheet name="all_data" sheetId="1" r:id="rId1"/>
@@ -69385,7 +69385,7 @@
     </row>
     <row r="57" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
-        <v>379</v>
+        <v>168</v>
       </c>
       <c r="B57" t="s">
         <v>289</v>
@@ -72687,7 +72687,7 @@
     </row>
     <row r="184" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A184" t="s">
-        <v>1680</v>
+        <v>178</v>
       </c>
       <c r="B184" t="s">
         <v>1681</v>

</xml_diff>